<commit_message>
Update IPL fantasy points
</commit_message>
<xml_diff>
--- a/outputs/owner_points_summary.xlsx
+++ b/outputs/owner_points_summary.xlsx
@@ -448,10 +448,10 @@
         <v>3073</v>
       </c>
       <c r="C2" t="n">
-        <v>3297</v>
+        <v>3171</v>
       </c>
       <c r="D2" t="n">
-        <v>6370</v>
+        <v>6244</v>
       </c>
     </row>
     <row r="3">
@@ -464,10 +464,10 @@
         <v>3474</v>
       </c>
       <c r="C3" t="n">
-        <v>3096</v>
+        <v>2852</v>
       </c>
       <c r="D3" t="n">
-        <v>6570</v>
+        <v>6326</v>
       </c>
     </row>
     <row r="4">
@@ -480,10 +480,10 @@
         <v>3193</v>
       </c>
       <c r="C4" t="n">
-        <v>4291</v>
+        <v>4140</v>
       </c>
       <c r="D4" t="n">
-        <v>7484</v>
+        <v>7333</v>
       </c>
     </row>
     <row r="5">
@@ -496,10 +496,10 @@
         <v>3063</v>
       </c>
       <c r="C5" t="n">
-        <v>4223</v>
+        <v>3964</v>
       </c>
       <c r="D5" t="n">
-        <v>7286</v>
+        <v>7027</v>
       </c>
     </row>
     <row r="6">
@@ -512,10 +512,10 @@
         <v>3043</v>
       </c>
       <c r="C6" t="n">
-        <v>2233</v>
+        <v>2115</v>
       </c>
       <c r="D6" t="n">
-        <v>5276</v>
+        <v>5158</v>
       </c>
     </row>
     <row r="7">
@@ -528,10 +528,10 @@
         <v>4457</v>
       </c>
       <c r="C7" t="n">
-        <v>3872</v>
+        <v>3634</v>
       </c>
       <c r="D7" t="n">
-        <v>8329</v>
+        <v>8091</v>
       </c>
     </row>
     <row r="8">
@@ -544,10 +544,10 @@
         <v>3445</v>
       </c>
       <c r="C8" t="n">
-        <v>3811</v>
+        <v>3441</v>
       </c>
       <c r="D8" t="n">
-        <v>7256</v>
+        <v>6886</v>
       </c>
     </row>
   </sheetData>

</xml_diff>